<commit_message>
fix(dashboard): resolve 500 error in weekly audit generation by supporting multiple broker variants and safe exception handling
</commit_message>
<xml_diff>
--- a/reports/weekly/2026_W36/report.xlsx
+++ b/reports/weekly/2026_W36/report.xlsx
@@ -9,7 +9,9 @@
   <sheets>
     <sheet name="Resumen Ejecutivo" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Trade Ledger" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Drift Tracker" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Reconciliation" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Equity Series" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Drift Tracker" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -415,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -438,102 +440,106 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>audit_2026_W36_1788381382</t>
+          <t>audit_2026_W36_1788383112</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Generado</t>
+          <t>Schema Version</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-02T20:36:22.678146+00:00</t>
+          <t>1.0.0</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Git Commit SHA</t>
+          <t>Generado</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1ad3f3fb4b813984961349a5b587b84642c46ae9</t>
+          <t>2026-09-02T21:05:12.866664+00:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Config Hash</t>
+          <t>Git Commit SHA</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>12c68c1a40b27329cb63cea9a38dcd9904875780ab5d4fae605308633eeb6a83</t>
+          <t>4040a27adfed0cb696c79cfb1e42b4e9c9c9c5b2</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Config Hash</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>12c68c1a40b27329cb63cea9a38dcd9904875780ab5d4fae605308633eeb6a83</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>Integrity Hash SHA256</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>646523772613458a016d6c1b1345a4ddf77ae1c08b1795b6115cc7271c594721</t>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>1946a275f4cef1491170eabd43b43dac15eecd72c871a5e16b88b979ce94221a</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Capital Inicial (USD)</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Patrimonio Actual (USD)</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>25</v>
+          <t>Reconciliation Status</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>PASS / 0 inconsistencies</t>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>PnL Neto Acumulado (USD)</t>
+          <t>Capital Inicial (USD)</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Profit Factor</t>
+          <t>Patrimonio Actual (USD)</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Win Rate (%)</t>
+          <t>PnL Neto Acumulado (USD)</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -543,7 +549,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Average R</t>
+          <t>Profit Factor</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -553,11 +559,31 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>Win Rate (%)</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Average R</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>Max Drawdown (%)</t>
         </is>
       </c>
-      <c r="B15" t="n">
-        <v>75</v>
+      <c r="B17" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -571,7 +597,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:P1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -587,65 +613,70 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>Entry Time</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Fill Price</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Stop Loss</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Take Profit</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Exit Time</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Exit Price</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Exit Reason</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Gross PnL</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Fees</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Net PnL</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>R Multiple</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Duration (Hours)</t>
         </is>
@@ -662,6 +693,254 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Check / Métrica</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Resultado / Conteo</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Status General</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Inconsistencias Totales</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>signals_orders_reconciled</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>orders_fills_reconciled</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>fills_positions_reconciled</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>positions_pnl_reconciled</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>risk_events_state_reconciled</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>orphan_events_count</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>missing_fills_count</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>duplicate_ids_count</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>inconsistent_states_count</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>pnl_mismatches_count</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Timestamp</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Equity (USD)</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Daily DD (%)</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Peak DD (%)</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>BTC Price</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>SOL Price</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-08-26T21:05:12.866664+00:00</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>100</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>60000</v>
+      </c>
+      <c r="F2" t="n">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-09-02T21:05:12.866664+00:00</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>100</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>61000</v>
+      </c>
+      <c r="F3" t="n">
+        <v>145</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -792,19 +1071,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="C6" t="n">
         <v>17.13</v>
       </c>
       <c r="D6" t="n">
-        <v>57.87</v>
+        <v>-17.13</v>
       </c>
       <c r="E6" t="n">
         <v>20.66</v>
       </c>
       <c r="F6" t="n">
-        <v>54.34</v>
+        <v>-20.66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(weekly-audit): add auto-download in UI, posix paths, and robust open_positions handling
</commit_message>
<xml_diff>
--- a/reports/weekly/2026_W36/report.xlsx
+++ b/reports/weekly/2026_W36/report.xlsx
@@ -440,7 +440,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>audit_2026_W36_1788383112</t>
+          <t>audit_2026_W36_1788383381</t>
         </is>
       </c>
     </row>
@@ -464,7 +464,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-02T21:05:12.866664+00:00</t>
+          <t>2026-09-02T21:09:41.227731+00:00</t>
         </is>
       </c>
     </row>
@@ -476,7 +476,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>4040a27adfed0cb696c79cfb1e42b4e9c9c9c5b2</t>
+          <t>5590913276524a1a5a404b42719358fd1daf9aca</t>
         </is>
       </c>
     </row>
@@ -500,7 +500,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>1946a275f4cef1491170eabd43b43dac15eecd72c871a5e16b88b979ce94221a</t>
+          <t>c432259023db59602206a2c011ec2679fa10ae370117e6f8671b3f41d86d6347</t>
         </is>
       </c>
     </row>
@@ -889,7 +889,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-26T21:05:12.866664+00:00</t>
+          <t>2026-08-26T21:09:41.227731+00:00</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -911,7 +911,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-02T21:05:12.866664+00:00</t>
+          <t>2026-09-02T21:09:41.227731+00:00</t>
         </is>
       </c>
       <c r="B3" t="n">

</xml_diff>